<commit_message>
WIP: scripts de analisis de gaps en proceso
</commit_message>
<xml_diff>
--- a/exports/historical-tariffs-ready.xlsx
+++ b/exports/historical-tariffs-ready.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H94"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1460,10 +1460,10 @@
         <v>2025-03-01</v>
       </c>
       <c r="F41" t="str">
-        <v>2025-07-31</v>
+        <v>2025-08-31</v>
       </c>
       <c r="G41" t="str">
-        <v>2025-03 = $20000.00</v>
+        <v>2025-03 = $20000.00 | 2025-08 = $20000.00</v>
       </c>
       <c r="H41" t="str">
         <v/>
@@ -1471,25 +1471,25 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>a12f5acf-4754-479a-853c-15926c2dac92</v>
+        <v>06f93e1a-5cc0-4741-8ad6-813745ea389d</v>
       </c>
       <c r="B42" t="str">
-        <v>Ladys Tango - Gabriela P.</v>
+        <v>Ladys Kizz</v>
       </c>
       <c r="C42" t="str">
-        <v>Histórica - Ladys Tango - Gabriela P. - 2025 - $7.500</v>
+        <v>Histórica - Ladys Kizz - 2025 - $30.000</v>
       </c>
       <c r="D42" t="str">
-        <v>7500.00</v>
+        <v>30000.00</v>
       </c>
       <c r="E42" t="str">
-        <v>2025-02-01</v>
+        <v>2025-09-01</v>
       </c>
       <c r="F42" t="str">
-        <v>2025-02-28</v>
+        <v>2025-11-30</v>
       </c>
       <c r="G42" t="str">
-        <v>2025-02 = $7500.00</v>
+        <v>2025-09 = $30000.00</v>
       </c>
       <c r="H42" t="str">
         <v/>
@@ -1497,25 +1497,25 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>a12f5acf-4754-479a-853c-15926c2dac92</v>
+        <v>06f93e1a-5cc0-4741-8ad6-813745ea389d</v>
       </c>
       <c r="B43" t="str">
-        <v>Ladys Tango - Gabriela P.</v>
+        <v>Ladys Kizz</v>
       </c>
       <c r="C43" t="str">
-        <v>Histórica - Ladys Tango - Gabriela P. - 2025 - $10.000</v>
+        <v>Histórica - Ladys Kizz - 2026 - $30.000</v>
       </c>
       <c r="D43" t="str">
-        <v>10000.00</v>
+        <v>30000.00</v>
       </c>
       <c r="E43" t="str">
-        <v>2025-03-01</v>
+        <v>2026-01-01</v>
       </c>
       <c r="F43" t="str">
-        <v>2025-04-30</v>
+        <v>2026-06-30</v>
       </c>
       <c r="G43" t="str">
-        <v>2025-03 = $10000.00</v>
+        <v>2026-01 = $30000.00</v>
       </c>
       <c r="H43" t="str">
         <v/>
@@ -1523,25 +1523,25 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>a12f5acf-4754-479a-853c-15926c2dac92</v>
+        <v>06f93e1a-5cc0-4741-8ad6-813745ea389d</v>
       </c>
       <c r="B44" t="str">
-        <v>Ladys Tango - Gabriela P.</v>
+        <v>Ladys Kizz</v>
       </c>
       <c r="C44" t="str">
-        <v>Histórica - Ladys Tango - Gabriela P. - 2025 - $11.000</v>
+        <v>Histórica - Ladys Kizz - 2026 - $15.000</v>
       </c>
       <c r="D44" t="str">
-        <v>11000.00</v>
+        <v>15000.00</v>
       </c>
       <c r="E44" t="str">
-        <v>2025-05-01</v>
+        <v>2026-07-01</v>
       </c>
       <c r="F44" t="str">
-        <v>2025-06-30</v>
+        <v>2026-07-31</v>
       </c>
       <c r="G44" t="str">
-        <v>2025-05 = $11000.00</v>
+        <v>2026-07 = $15000.00</v>
       </c>
       <c r="H44" t="str">
         <v/>
@@ -1549,25 +1549,25 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>a12f5acf-4754-479a-853c-15926c2dac92</v>
+        <v>06f93e1a-5cc0-4741-8ad6-813745ea389d</v>
       </c>
       <c r="B45" t="str">
-        <v>Ladys Tango - Gabriela P.</v>
+        <v>Ladys Kizz</v>
       </c>
       <c r="C45" t="str">
-        <v>Histórica - Ladys Tango - Gabriela P. - 2025 - $20.000</v>
+        <v>Histórica - Ladys Kizz - 2026 - $40.000</v>
       </c>
       <c r="D45" t="str">
-        <v>20000.00</v>
+        <v>40000.00</v>
       </c>
       <c r="E45" t="str">
-        <v>2025-07-01</v>
+        <v>2026-08-01</v>
       </c>
       <c r="F45" t="str">
-        <v>2025-07-31</v>
+        <v>2026-08-31</v>
       </c>
       <c r="G45" t="str">
-        <v>2025-07 = $20000.00</v>
+        <v>2026-08 = $40000.00</v>
       </c>
       <c r="H45" t="str">
         <v/>
@@ -1575,25 +1575,25 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>b96017bd-9ee1-4bde-ad35-ad961a78e5f5</v>
+        <v>a12f5acf-4754-479a-853c-15926c2dac92</v>
       </c>
       <c r="B46" t="str">
-        <v>Mambo en parejas</v>
+        <v>Ladys Tango - Gabriela P.</v>
       </c>
       <c r="C46" t="str">
-        <v>Histórica - Mambo en parejas - 2026 - $15.000</v>
+        <v>Histórica - Ladys Tango - Gabriela P. - 2025 - $7.500</v>
       </c>
       <c r="D46" t="str">
-        <v>15000.00</v>
+        <v>7500.00</v>
       </c>
       <c r="E46" t="str">
-        <v>2026-02-01</v>
+        <v>2025-02-01</v>
       </c>
       <c r="F46" t="str">
-        <v>2026-02-28</v>
+        <v>2025-02-28</v>
       </c>
       <c r="G46" t="str">
-        <v>2026-02 = $15000.00</v>
+        <v>2025-02 = $7500.00</v>
       </c>
       <c r="H46" t="str">
         <v/>
@@ -1601,51 +1601,51 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>b96017bd-9ee1-4bde-ad35-ad961a78e5f5</v>
+        <v>a12f5acf-4754-479a-853c-15926c2dac92</v>
       </c>
       <c r="B47" t="str">
-        <v>Mambo en parejas</v>
+        <v>Ladys Tango - Gabriela P.</v>
       </c>
       <c r="C47" t="str">
-        <v>Histórica - Mambo en parejas - 2026 - $30.000</v>
+        <v>Histórica - Ladys Tango - Gabriela P. - 2025 - $10.000</v>
       </c>
       <c r="D47" t="str">
-        <v>30000.00</v>
+        <v>10000.00</v>
       </c>
       <c r="E47" t="str">
-        <v>2026-03-01</v>
+        <v>2025-03-01</v>
       </c>
       <c r="F47" t="str">
-        <v>2026-07-31</v>
+        <v>2025-04-30</v>
       </c>
       <c r="G47" t="str">
-        <v>2026-03 = $30000.00 | 2026-05 = $30000.00</v>
+        <v>2025-03 = $10000.00</v>
       </c>
       <c r="H47" t="str">
-        <v>2026-07 ($15000.00)</v>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>b96017bd-9ee1-4bde-ad35-ad961a78e5f5</v>
+        <v>a12f5acf-4754-479a-853c-15926c2dac92</v>
       </c>
       <c r="B48" t="str">
-        <v>Mambo en parejas</v>
+        <v>Ladys Tango - Gabriela P.</v>
       </c>
       <c r="C48" t="str">
-        <v>Histórica - Mambo en parejas - 2026 - $40.000</v>
+        <v>Histórica - Ladys Tango - Gabriela P. - 2025 - $11.000</v>
       </c>
       <c r="D48" t="str">
-        <v>40000.00</v>
+        <v>11000.00</v>
       </c>
       <c r="E48" t="str">
-        <v>2026-08-01</v>
+        <v>2025-05-01</v>
       </c>
       <c r="F48" t="str">
-        <v>2026-08-31</v>
+        <v>2025-06-30</v>
       </c>
       <c r="G48" t="str">
-        <v>2026-08 = $40000.00</v>
+        <v>2025-05 = $11000.00</v>
       </c>
       <c r="H48" t="str">
         <v/>
@@ -1653,25 +1653,25 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>1a8e1c0e-1f96-4de2-a33d-c932e74f2314</v>
+        <v>a12f5acf-4754-479a-853c-15926c2dac92</v>
       </c>
       <c r="B49" t="str">
-        <v>Ritmos latinos y caribeños</v>
+        <v>Ladys Tango - Gabriela P.</v>
       </c>
       <c r="C49" t="str">
-        <v>Histórica - Ritmos latinos y caribeños - 2025 - $15.000</v>
+        <v>Histórica - Ladys Tango - Gabriela P. - 2025 - $20.000</v>
       </c>
       <c r="D49" t="str">
-        <v>15000.00</v>
+        <v>20000.00</v>
       </c>
       <c r="E49" t="str">
-        <v>2025-02-01</v>
+        <v>2025-07-01</v>
       </c>
       <c r="F49" t="str">
-        <v>2025-02-28</v>
+        <v>2025-07-31</v>
       </c>
       <c r="G49" t="str">
-        <v>2025-02 = $15000.00</v>
+        <v>2025-07 = $20000.00</v>
       </c>
       <c r="H49" t="str">
         <v/>
@@ -1679,25 +1679,25 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>1a8e1c0e-1f96-4de2-a33d-c932e74f2314</v>
+        <v>b96017bd-9ee1-4bde-ad35-ad961a78e5f5</v>
       </c>
       <c r="B50" t="str">
-        <v>Ritmos latinos y caribeños</v>
+        <v>Mambo en parejas</v>
       </c>
       <c r="C50" t="str">
-        <v>Histórica - Ritmos latinos y caribeños - 2025 - $20.000</v>
+        <v>Histórica - Mambo en parejas - 2026 - $15.000</v>
       </c>
       <c r="D50" t="str">
-        <v>20000.00</v>
+        <v>15000.00</v>
       </c>
       <c r="E50" t="str">
-        <v>2025-03-01</v>
+        <v>2026-02-01</v>
       </c>
       <c r="F50" t="str">
-        <v>2025-07-31</v>
+        <v>2026-02-28</v>
       </c>
       <c r="G50" t="str">
-        <v>2025-03 = $20000.00</v>
+        <v>2026-02 = $15000.00</v>
       </c>
       <c r="H50" t="str">
         <v/>
@@ -1705,51 +1705,51 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>71bc486f-8a3d-46bb-a102-838cfef0a1fc</v>
+        <v>b96017bd-9ee1-4bde-ad35-ad961a78e5f5</v>
       </c>
       <c r="B51" t="str">
-        <v>S.C Adultos (+18 años)</v>
+        <v>Mambo en parejas</v>
       </c>
       <c r="C51" t="str">
-        <v>Histórica - S.C Adultos (+18 años) - 2025 - $15.000</v>
+        <v>Histórica - Mambo en parejas - 2026 - $30.000</v>
       </c>
       <c r="D51" t="str">
-        <v>15000.00</v>
+        <v>30000.00</v>
       </c>
       <c r="E51" t="str">
-        <v>2025-02-01</v>
+        <v>2026-03-01</v>
       </c>
       <c r="F51" t="str">
-        <v>2025-02-28</v>
+        <v>2026-07-31</v>
       </c>
       <c r="G51" t="str">
-        <v>2025-02 = $15000.00</v>
+        <v>2026-03 = $30000.00 | 2026-05 = $30000.00</v>
       </c>
       <c r="H51" t="str">
-        <v/>
+        <v>2026-07 ($15000.00)</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>71bc486f-8a3d-46bb-a102-838cfef0a1fc</v>
+        <v>b96017bd-9ee1-4bde-ad35-ad961a78e5f5</v>
       </c>
       <c r="B52" t="str">
-        <v>S.C Adultos (+18 años)</v>
+        <v>Mambo en parejas</v>
       </c>
       <c r="C52" t="str">
-        <v>Histórica - S.C Adultos (+18 años) - 2025 - $20.000</v>
+        <v>Histórica - Mambo en parejas - 2026 - $40.000</v>
       </c>
       <c r="D52" t="str">
-        <v>20000.00</v>
+        <v>40000.00</v>
       </c>
       <c r="E52" t="str">
-        <v>2025-03-01</v>
+        <v>2026-08-01</v>
       </c>
       <c r="F52" t="str">
-        <v>2025-04-30</v>
+        <v>2026-08-31</v>
       </c>
       <c r="G52" t="str">
-        <v>2025-03 = $20000.00</v>
+        <v>2026-08 = $40000.00</v>
       </c>
       <c r="H52" t="str">
         <v/>
@@ -1757,13 +1757,13 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>4b2663bf-5ab4-42e5-865c-2af4da2cf5ff</v>
+        <v>1a8e1c0e-1f96-4de2-a33d-c932e74f2314</v>
       </c>
       <c r="B53" t="str">
-        <v>S.C Infantil (6-11 años)</v>
+        <v>Ritmos latinos y caribeños</v>
       </c>
       <c r="C53" t="str">
-        <v>Histórica - S.C Infantil (6-11 años) - 2025 - $15.000</v>
+        <v>Histórica - Ritmos latinos y caribeños - 2025 - $15.000</v>
       </c>
       <c r="D53" t="str">
         <v>15000.00</v>
@@ -1783,13 +1783,13 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>4b2663bf-5ab4-42e5-865c-2af4da2cf5ff</v>
+        <v>1a8e1c0e-1f96-4de2-a33d-c932e74f2314</v>
       </c>
       <c r="B54" t="str">
-        <v>S.C Infantil (6-11 años)</v>
+        <v>Ritmos latinos y caribeños</v>
       </c>
       <c r="C54" t="str">
-        <v>Histórica - S.C Infantil (6-11 años) - 2025 - $20.000</v>
+        <v>Histórica - Ritmos latinos y caribeños - 2025 - $20.000</v>
       </c>
       <c r="D54" t="str">
         <v>20000.00</v>
@@ -1798,7 +1798,7 @@
         <v>2025-03-01</v>
       </c>
       <c r="F54" t="str">
-        <v>2025-04-30</v>
+        <v>2025-07-31</v>
       </c>
       <c r="G54" t="str">
         <v>2025-03 = $20000.00</v>
@@ -1809,13 +1809,13 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>f8a32bf2-9e2a-48b5-9f2e-a8b9da860fb3</v>
+        <v>71bc486f-8a3d-46bb-a102-838cfef0a1fc</v>
       </c>
       <c r="B55" t="str">
-        <v>S.C Juvenil (12-17 años)</v>
+        <v>S.C Adultos (+18 años)</v>
       </c>
       <c r="C55" t="str">
-        <v>Histórica - S.C Juvenil (12-17 años) - 2025 - $15.000</v>
+        <v>Histórica - S.C Adultos (+18 años) - 2025 - $15.000</v>
       </c>
       <c r="D55" t="str">
         <v>15000.00</v>
@@ -1835,13 +1835,13 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>f8a32bf2-9e2a-48b5-9f2e-a8b9da860fb3</v>
+        <v>71bc486f-8a3d-46bb-a102-838cfef0a1fc</v>
       </c>
       <c r="B56" t="str">
-        <v>S.C Juvenil (12-17 años)</v>
+        <v>S.C Adultos (+18 años)</v>
       </c>
       <c r="C56" t="str">
-        <v>Histórica - S.C Juvenil (12-17 años) - 2025 - $20.000</v>
+        <v>Histórica - S.C Adultos (+18 años) - 2025 - $20.000</v>
       </c>
       <c r="D56" t="str">
         <v>20000.00</v>
@@ -1850,10 +1850,10 @@
         <v>2025-03-01</v>
       </c>
       <c r="F56" t="str">
-        <v>2025-04-30</v>
+        <v>2025-08-31</v>
       </c>
       <c r="G56" t="str">
-        <v>2025-03 = $20000.00</v>
+        <v>2025-03 = $20000.00 | 2025-05 = $20000.00</v>
       </c>
       <c r="H56" t="str">
         <v/>
@@ -1861,25 +1861,25 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>dd4b0323-e82f-4b02-89c0-0f8e520033ed</v>
+        <v>71bc486f-8a3d-46bb-a102-838cfef0a1fc</v>
       </c>
       <c r="B57" t="str">
-        <v>Street Int/Avanzado</v>
+        <v>S.C Adultos (+18 años)</v>
       </c>
       <c r="C57" t="str">
-        <v>Histórica - Street Int/Avanzado - 2025 - $15.000</v>
+        <v>Histórica - S.C Adultos (+18 años) - 2025 - $30.000</v>
       </c>
       <c r="D57" t="str">
-        <v>15000.00</v>
+        <v>30000.00</v>
       </c>
       <c r="E57" t="str">
-        <v>2025-02-01</v>
+        <v>2025-09-01</v>
       </c>
       <c r="F57" t="str">
-        <v>2025-02-28</v>
+        <v>2025-11-30</v>
       </c>
       <c r="G57" t="str">
-        <v>2025-02 = $15000.00</v>
+        <v>2025-09 = $30000.00</v>
       </c>
       <c r="H57" t="str">
         <v/>
@@ -1887,25 +1887,25 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>dd4b0323-e82f-4b02-89c0-0f8e520033ed</v>
+        <v>71bc486f-8a3d-46bb-a102-838cfef0a1fc</v>
       </c>
       <c r="B58" t="str">
-        <v>Street Int/Avanzado</v>
+        <v>S.C Adultos (+18 años)</v>
       </c>
       <c r="C58" t="str">
-        <v>Histórica - Street Int/Avanzado - 2025 - $20.000</v>
+        <v>Histórica - S.C Adultos (+18 años) - 2026 - $30.000</v>
       </c>
       <c r="D58" t="str">
-        <v>20000.00</v>
+        <v>30000.00</v>
       </c>
       <c r="E58" t="str">
-        <v>2025-03-01</v>
+        <v>2026-01-01</v>
       </c>
       <c r="F58" t="str">
-        <v>2025-04-30</v>
+        <v>2026-06-30</v>
       </c>
       <c r="G58" t="str">
-        <v>2025-03 = $20000.00</v>
+        <v>2026-01 = $30000.00</v>
       </c>
       <c r="H58" t="str">
         <v/>
@@ -1913,25 +1913,25 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
+        <v>71bc486f-8a3d-46bb-a102-838cfef0a1fc</v>
       </c>
       <c r="B59" t="str">
-        <v>Tango (Inter/Avanz)</v>
+        <v>S.C Adultos (+18 años)</v>
       </c>
       <c r="C59" t="str">
-        <v>Histórica - Tango (Inter/Avanz) - 2025 - $15.000</v>
+        <v>Histórica - S.C Adultos (+18 años) - 2026 - $15.000</v>
       </c>
       <c r="D59" t="str">
         <v>15000.00</v>
       </c>
       <c r="E59" t="str">
-        <v>2025-02-01</v>
+        <v>2026-07-01</v>
       </c>
       <c r="F59" t="str">
-        <v>2025-02-28</v>
+        <v>2026-07-31</v>
       </c>
       <c r="G59" t="str">
-        <v>2025-02 = $15000.00</v>
+        <v>2026-07 = $15000.00</v>
       </c>
       <c r="H59" t="str">
         <v/>
@@ -1939,25 +1939,25 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
+        <v>71bc486f-8a3d-46bb-a102-838cfef0a1fc</v>
       </c>
       <c r="B60" t="str">
-        <v>Tango (Inter/Avanz)</v>
+        <v>S.C Adultos (+18 años)</v>
       </c>
       <c r="C60" t="str">
-        <v>Histórica - Tango (Inter/Avanz) - 2025 - $20.000</v>
+        <v>Histórica - S.C Adultos (+18 años) - 2026 - $40.000</v>
       </c>
       <c r="D60" t="str">
-        <v>20000.00</v>
+        <v>40000.00</v>
       </c>
       <c r="E60" t="str">
-        <v>2025-03-01</v>
+        <v>2026-08-01</v>
       </c>
       <c r="F60" t="str">
-        <v>2025-08-31</v>
+        <v>2026-08-31</v>
       </c>
       <c r="G60" t="str">
-        <v>2025-03 = $20000.00</v>
+        <v>2026-08 = $40000.00</v>
       </c>
       <c r="H60" t="str">
         <v/>
@@ -1965,25 +1965,25 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
+        <v>4b2663bf-5ab4-42e5-865c-2af4da2cf5ff</v>
       </c>
       <c r="B61" t="str">
-        <v>Tango (Inter/Avanz)</v>
+        <v>S.C Infantil (6-11 años)</v>
       </c>
       <c r="C61" t="str">
-        <v>Histórica - Tango (Inter/Avanz) - 2025 - $30.000</v>
+        <v>Histórica - S.C Infantil (6-11 años) - 2025 - $15.000</v>
       </c>
       <c r="D61" t="str">
-        <v>30000.00</v>
+        <v>15000.00</v>
       </c>
       <c r="E61" t="str">
-        <v>2025-09-01</v>
+        <v>2025-02-01</v>
       </c>
       <c r="F61" t="str">
-        <v>2025-11-30</v>
+        <v>2025-02-28</v>
       </c>
       <c r="G61" t="str">
-        <v>2025-09 = $30000.00</v>
+        <v>2025-02 = $15000.00</v>
       </c>
       <c r="H61" t="str">
         <v/>
@@ -1991,51 +1991,51 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
+        <v>4b2663bf-5ab4-42e5-865c-2af4da2cf5ff</v>
       </c>
       <c r="B62" t="str">
-        <v>Tango (Inter/Avanz)</v>
+        <v>S.C Infantil (6-11 años)</v>
       </c>
       <c r="C62" t="str">
-        <v>Histórica - Tango (Inter/Avanz) - 2026 - $30.000</v>
+        <v>Histórica - S.C Infantil (6-11 años) - 2025 - $20.000</v>
       </c>
       <c r="D62" t="str">
-        <v>30000.00</v>
+        <v>20000.00</v>
       </c>
       <c r="E62" t="str">
-        <v>2026-03-01</v>
+        <v>2025-03-01</v>
       </c>
       <c r="F62" t="str">
-        <v>2026-07-31</v>
+        <v>2025-08-31</v>
       </c>
       <c r="G62" t="str">
-        <v>2026-03 = $30000.00 | 2026-05 = $30000.00</v>
+        <v>2025-03 = $20000.00 | 2025-05 = $20000.00</v>
       </c>
       <c r="H62" t="str">
-        <v>2026-07 ($15000.00)</v>
+        <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
+        <v>4b2663bf-5ab4-42e5-865c-2af4da2cf5ff</v>
       </c>
       <c r="B63" t="str">
-        <v>Tango (Inter/Avanz)</v>
+        <v>S.C Infantil (6-11 años)</v>
       </c>
       <c r="C63" t="str">
-        <v>Histórica - Tango (Inter/Avanz) - 2026 - $40.000</v>
+        <v>Histórica - S.C Infantil (6-11 años) - 2025 - $30.000</v>
       </c>
       <c r="D63" t="str">
-        <v>40000.00</v>
+        <v>30000.00</v>
       </c>
       <c r="E63" t="str">
-        <v>2026-08-01</v>
+        <v>2025-09-01</v>
       </c>
       <c r="F63" t="str">
-        <v>2026-08-31</v>
+        <v>2025-11-30</v>
       </c>
       <c r="G63" t="str">
-        <v>2026-08 = $40000.00</v>
+        <v>2025-09 = $30000.00</v>
       </c>
       <c r="H63" t="str">
         <v/>
@@ -2043,25 +2043,25 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>23888530-c53d-4c40-94ee-982518e5d2f6</v>
+        <v>4b2663bf-5ab4-42e5-865c-2af4da2cf5ff</v>
       </c>
       <c r="B64" t="str">
-        <v>Tango Inicial</v>
+        <v>S.C Infantil (6-11 años)</v>
       </c>
       <c r="C64" t="str">
-        <v>Histórica - Tango Inicial - 2026 - $30.000</v>
+        <v>Histórica - S.C Infantil (6-11 años) - 2026 - $30.000</v>
       </c>
       <c r="D64" t="str">
         <v>30000.00</v>
       </c>
       <c r="E64" t="str">
-        <v>2026-03-01</v>
+        <v>2026-01-01</v>
       </c>
       <c r="F64" t="str">
-        <v>2026-03-31</v>
+        <v>2026-06-30</v>
       </c>
       <c r="G64" t="str">
-        <v>2026-03 = $30000.00</v>
+        <v>2026-01 = $30000.00</v>
       </c>
       <c r="H64" t="str">
         <v/>
@@ -2069,25 +2069,25 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+        <v>4b2663bf-5ab4-42e5-865c-2af4da2cf5ff</v>
       </c>
       <c r="B65" t="str">
-        <v>Teens (8 a 12 años)</v>
+        <v>S.C Infantil (6-11 años)</v>
       </c>
       <c r="C65" t="str">
-        <v>Histórica - Teens (8 a 12 años) - 2025 - $15.000</v>
+        <v>Histórica - S.C Infantil (6-11 años) - 2026 - $15.000</v>
       </c>
       <c r="D65" t="str">
         <v>15000.00</v>
       </c>
       <c r="E65" t="str">
-        <v>2025-02-01</v>
+        <v>2026-07-01</v>
       </c>
       <c r="F65" t="str">
-        <v>2025-02-28</v>
+        <v>2026-07-31</v>
       </c>
       <c r="G65" t="str">
-        <v>2025-02 = $15000.00</v>
+        <v>2026-07 = $15000.00</v>
       </c>
       <c r="H65" t="str">
         <v/>
@@ -2095,25 +2095,25 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+        <v>4b2663bf-5ab4-42e5-865c-2af4da2cf5ff</v>
       </c>
       <c r="B66" t="str">
-        <v>Teens (8 a 12 años)</v>
+        <v>S.C Infantil (6-11 años)</v>
       </c>
       <c r="C66" t="str">
-        <v>Histórica - Teens (8 a 12 años) - 2025 - $20.000</v>
+        <v>Histórica - S.C Infantil (6-11 años) - 2026 - $40.000</v>
       </c>
       <c r="D66" t="str">
-        <v>20000.00</v>
+        <v>40000.00</v>
       </c>
       <c r="E66" t="str">
-        <v>2025-03-01</v>
+        <v>2026-08-01</v>
       </c>
       <c r="F66" t="str">
-        <v>2025-08-31</v>
+        <v>2026-08-31</v>
       </c>
       <c r="G66" t="str">
-        <v>2025-03 = $20000.00</v>
+        <v>2026-08 = $40000.00</v>
       </c>
       <c r="H66" t="str">
         <v/>
@@ -2121,25 +2121,25 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+        <v>f8a32bf2-9e2a-48b5-9f2e-a8b9da860fb3</v>
       </c>
       <c r="B67" t="str">
-        <v>Teens (8 a 12 años)</v>
+        <v>S.C Juvenil (12-17 años)</v>
       </c>
       <c r="C67" t="str">
-        <v>Histórica - Teens (8 a 12 años) - 2025 - $30.000</v>
+        <v>Histórica - S.C Juvenil (12-17 años) - 2025 - $15.000</v>
       </c>
       <c r="D67" t="str">
-        <v>30000.00</v>
+        <v>15000.00</v>
       </c>
       <c r="E67" t="str">
-        <v>2025-09-01</v>
+        <v>2025-02-01</v>
       </c>
       <c r="F67" t="str">
-        <v>2025-10-31</v>
+        <v>2025-02-28</v>
       </c>
       <c r="G67" t="str">
-        <v>2025-09 = $30000.00</v>
+        <v>2025-02 = $15000.00</v>
       </c>
       <c r="H67" t="str">
         <v/>
@@ -2147,25 +2147,25 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+        <v>f8a32bf2-9e2a-48b5-9f2e-a8b9da860fb3</v>
       </c>
       <c r="B68" t="str">
-        <v>Teens (8 a 12 años)</v>
+        <v>S.C Juvenil (12-17 años)</v>
       </c>
       <c r="C68" t="str">
-        <v>Histórica - Teens (8 a 12 años) - 2025 - $25.000</v>
+        <v>Histórica - S.C Juvenil (12-17 años) - 2025 - $20.000</v>
       </c>
       <c r="D68" t="str">
-        <v>25000.00</v>
+        <v>20000.00</v>
       </c>
       <c r="E68" t="str">
-        <v>2025-11-01</v>
+        <v>2025-03-01</v>
       </c>
       <c r="F68" t="str">
-        <v>2025-11-30</v>
+        <v>2025-08-31</v>
       </c>
       <c r="G68" t="str">
-        <v>2025-11 = $25000.00</v>
+        <v>2025-03 = $20000.00 | 2025-05 = $20000.00</v>
       </c>
       <c r="H68" t="str">
         <v/>
@@ -2173,25 +2173,25 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+        <v>f8a32bf2-9e2a-48b5-9f2e-a8b9da860fb3</v>
       </c>
       <c r="B69" t="str">
-        <v>Teens (8 a 12 años)</v>
+        <v>S.C Juvenil (12-17 años)</v>
       </c>
       <c r="C69" t="str">
-        <v>Histórica - Teens (8 a 12 años) - 2026 - $30.000</v>
+        <v>Histórica - S.C Juvenil (12-17 años) - 2025 - $30.000</v>
       </c>
       <c r="D69" t="str">
         <v>30000.00</v>
       </c>
       <c r="E69" t="str">
-        <v>2026-01-01</v>
+        <v>2025-09-01</v>
       </c>
       <c r="F69" t="str">
-        <v>2026-01-31</v>
+        <v>2025-11-30</v>
       </c>
       <c r="G69" t="str">
-        <v>2026-01 = $30000.00</v>
+        <v>2025-09 = $30000.00</v>
       </c>
       <c r="H69" t="str">
         <v/>
@@ -2199,25 +2199,25 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+        <v>f8a32bf2-9e2a-48b5-9f2e-a8b9da860fb3</v>
       </c>
       <c r="B70" t="str">
-        <v>Teens (8 a 12 años)</v>
+        <v>S.C Juvenil (12-17 años)</v>
       </c>
       <c r="C70" t="str">
-        <v>Histórica - Teens (8 a 12 años) - 2026 - $15.000</v>
+        <v>Histórica - S.C Juvenil (12-17 años) - 2026 - $30.000</v>
       </c>
       <c r="D70" t="str">
-        <v>15000.00</v>
+        <v>30000.00</v>
       </c>
       <c r="E70" t="str">
-        <v>2026-02-01</v>
+        <v>2026-01-01</v>
       </c>
       <c r="F70" t="str">
-        <v>2026-02-28</v>
+        <v>2026-06-30</v>
       </c>
       <c r="G70" t="str">
-        <v>2026-02 = $15000.00</v>
+        <v>2026-01 = $30000.00</v>
       </c>
       <c r="H70" t="str">
         <v/>
@@ -2225,39 +2225,39 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+        <v>f8a32bf2-9e2a-48b5-9f2e-a8b9da860fb3</v>
       </c>
       <c r="B71" t="str">
-        <v>Teens (8 a 12 años)</v>
+        <v>S.C Juvenil (12-17 años)</v>
       </c>
       <c r="C71" t="str">
-        <v>Histórica - Teens (8 a 12 años) - 2026 - $30.000</v>
+        <v>Histórica - S.C Juvenil (12-17 años) - 2026 - $15.000</v>
       </c>
       <c r="D71" t="str">
-        <v>30000.00</v>
+        <v>15000.00</v>
       </c>
       <c r="E71" t="str">
-        <v>2026-03-01</v>
+        <v>2026-07-01</v>
       </c>
       <c r="F71" t="str">
         <v>2026-07-31</v>
       </c>
       <c r="G71" t="str">
-        <v>2026-03 = $30000.00 | 2026-05 = $30000.00</v>
+        <v>2026-07 = $15000.00</v>
       </c>
       <c r="H71" t="str">
-        <v>2026-07 ($15000.00)</v>
+        <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+        <v>f8a32bf2-9e2a-48b5-9f2e-a8b9da860fb3</v>
       </c>
       <c r="B72" t="str">
-        <v>Teens (8 a 12 años)</v>
+        <v>S.C Juvenil (12-17 años)</v>
       </c>
       <c r="C72" t="str">
-        <v>Histórica - Teens (8 a 12 años) - 2026 - $40.000</v>
+        <v>Histórica - S.C Juvenil (12-17 años) - 2026 - $40.000</v>
       </c>
       <c r="D72" t="str">
         <v>40000.00</v>
@@ -2277,59 +2277,579 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>5e8e8fd7-a08b-4443-8ba0-30ee263ffa1b</v>
+        <v>dd4b0323-e82f-4b02-89c0-0f8e520033ed</v>
       </c>
       <c r="B73" t="str">
-        <v>Zumba - Profe Joselo</v>
+        <v>Street Int/Avanzado</v>
       </c>
       <c r="C73" t="str">
-        <v>Histórica - Zumba - Profe Joselo - 2026 - $30.000</v>
+        <v>Histórica - Street Int/Avanzado - 2025 - $15.000</v>
       </c>
       <c r="D73" t="str">
-        <v>30000.00</v>
+        <v>15000.00</v>
       </c>
       <c r="E73" t="str">
-        <v>2026-05-01</v>
+        <v>2025-02-01</v>
       </c>
       <c r="F73" t="str">
-        <v>2026-07-31</v>
+        <v>2025-02-28</v>
       </c>
       <c r="G73" t="str">
-        <v>2026-05 = $30000.00</v>
+        <v>2025-02 = $15000.00</v>
       </c>
       <c r="H73" t="str">
-        <v>2026-07 ($15000.00)</v>
+        <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
+        <v>dd4b0323-e82f-4b02-89c0-0f8e520033ed</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Street Int/Avanzado</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Histórica - Street Int/Avanzado - 2025 - $20.000</v>
+      </c>
+      <c r="D74" t="str">
+        <v>20000.00</v>
+      </c>
+      <c r="E74" t="str">
+        <v>2025-03-01</v>
+      </c>
+      <c r="F74" t="str">
+        <v>2025-08-31</v>
+      </c>
+      <c r="G74" t="str">
+        <v>2025-03 = $20000.00 | 2025-05 = $20000.00</v>
+      </c>
+      <c r="H74" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>dd4b0323-e82f-4b02-89c0-0f8e520033ed</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Street Int/Avanzado</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Histórica - Street Int/Avanzado - 2025 - $30.000</v>
+      </c>
+      <c r="D75" t="str">
+        <v>30000.00</v>
+      </c>
+      <c r="E75" t="str">
+        <v>2025-09-01</v>
+      </c>
+      <c r="F75" t="str">
+        <v>2025-11-30</v>
+      </c>
+      <c r="G75" t="str">
+        <v>2025-09 = $30000.00</v>
+      </c>
+      <c r="H75" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>dd4b0323-e82f-4b02-89c0-0f8e520033ed</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Street Int/Avanzado</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Histórica - Street Int/Avanzado - 2026 - $30.000</v>
+      </c>
+      <c r="D76" t="str">
+        <v>30000.00</v>
+      </c>
+      <c r="E76" t="str">
+        <v>2026-01-01</v>
+      </c>
+      <c r="F76" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="G76" t="str">
+        <v>2026-01 = $30000.00</v>
+      </c>
+      <c r="H76" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>dd4b0323-e82f-4b02-89c0-0f8e520033ed</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Street Int/Avanzado</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Histórica - Street Int/Avanzado - 2026 - $15.000</v>
+      </c>
+      <c r="D77" t="str">
+        <v>15000.00</v>
+      </c>
+      <c r="E77" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="F77" t="str">
+        <v>2026-07-31</v>
+      </c>
+      <c r="G77" t="str">
+        <v>2026-07 = $15000.00</v>
+      </c>
+      <c r="H77" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>dd4b0323-e82f-4b02-89c0-0f8e520033ed</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Street Int/Avanzado</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Histórica - Street Int/Avanzado - 2026 - $40.000</v>
+      </c>
+      <c r="D78" t="str">
+        <v>40000.00</v>
+      </c>
+      <c r="E78" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="F78" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G78" t="str">
+        <v>2026-08 = $40000.00</v>
+      </c>
+      <c r="H78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Tango (Inter/Avanz)</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Histórica - Tango (Inter/Avanz) - 2025 - $15.000</v>
+      </c>
+      <c r="D79" t="str">
+        <v>15000.00</v>
+      </c>
+      <c r="E79" t="str">
+        <v>2025-02-01</v>
+      </c>
+      <c r="F79" t="str">
+        <v>2025-02-28</v>
+      </c>
+      <c r="G79" t="str">
+        <v>2025-02 = $15000.00</v>
+      </c>
+      <c r="H79" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Tango (Inter/Avanz)</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Histórica - Tango (Inter/Avanz) - 2025 - $20.000</v>
+      </c>
+      <c r="D80" t="str">
+        <v>20000.00</v>
+      </c>
+      <c r="E80" t="str">
+        <v>2025-03-01</v>
+      </c>
+      <c r="F80" t="str">
+        <v>2025-08-31</v>
+      </c>
+      <c r="G80" t="str">
+        <v>2025-03 = $20000.00</v>
+      </c>
+      <c r="H80" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Tango (Inter/Avanz)</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Histórica - Tango (Inter/Avanz) - 2025 - $30.000</v>
+      </c>
+      <c r="D81" t="str">
+        <v>30000.00</v>
+      </c>
+      <c r="E81" t="str">
+        <v>2025-09-01</v>
+      </c>
+      <c r="F81" t="str">
+        <v>2025-11-30</v>
+      </c>
+      <c r="G81" t="str">
+        <v>2025-09 = $30000.00</v>
+      </c>
+      <c r="H81" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Tango (Inter/Avanz)</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Histórica - Tango (Inter/Avanz) - 2026 - $30.000</v>
+      </c>
+      <c r="D82" t="str">
+        <v>30000.00</v>
+      </c>
+      <c r="E82" t="str">
+        <v>2026-03-01</v>
+      </c>
+      <c r="F82" t="str">
+        <v>2026-07-31</v>
+      </c>
+      <c r="G82" t="str">
+        <v>2026-03 = $30000.00 | 2026-05 = $30000.00</v>
+      </c>
+      <c r="H82" t="str">
+        <v>2026-07 ($15000.00)</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Tango (Inter/Avanz)</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Histórica - Tango (Inter/Avanz) - 2026 - $40.000</v>
+      </c>
+      <c r="D83" t="str">
+        <v>40000.00</v>
+      </c>
+      <c r="E83" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="F83" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G83" t="str">
+        <v>2026-08 = $40000.00</v>
+      </c>
+      <c r="H83" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>23888530-c53d-4c40-94ee-982518e5d2f6</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Tango Inicial</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Histórica - Tango Inicial - 2026 - $30.000</v>
+      </c>
+      <c r="D84" t="str">
+        <v>30000.00</v>
+      </c>
+      <c r="E84" t="str">
+        <v>2026-03-01</v>
+      </c>
+      <c r="F84" t="str">
+        <v>2026-03-31</v>
+      </c>
+      <c r="G84" t="str">
+        <v>2026-03 = $30000.00</v>
+      </c>
+      <c r="H84" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Teens (8 a 12 años)</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Histórica - Teens (8 a 12 años) - 2025 - $15.000</v>
+      </c>
+      <c r="D85" t="str">
+        <v>15000.00</v>
+      </c>
+      <c r="E85" t="str">
+        <v>2025-02-01</v>
+      </c>
+      <c r="F85" t="str">
+        <v>2025-02-28</v>
+      </c>
+      <c r="G85" t="str">
+        <v>2025-02 = $15000.00</v>
+      </c>
+      <c r="H85" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Teens (8 a 12 años)</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Histórica - Teens (8 a 12 años) - 2025 - $20.000</v>
+      </c>
+      <c r="D86" t="str">
+        <v>20000.00</v>
+      </c>
+      <c r="E86" t="str">
+        <v>2025-03-01</v>
+      </c>
+      <c r="F86" t="str">
+        <v>2025-08-31</v>
+      </c>
+      <c r="G86" t="str">
+        <v>2025-03 = $20000.00</v>
+      </c>
+      <c r="H86" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Teens (8 a 12 años)</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Histórica - Teens (8 a 12 años) - 2025 - $30.000</v>
+      </c>
+      <c r="D87" t="str">
+        <v>30000.00</v>
+      </c>
+      <c r="E87" t="str">
+        <v>2025-09-01</v>
+      </c>
+      <c r="F87" t="str">
+        <v>2025-10-31</v>
+      </c>
+      <c r="G87" t="str">
+        <v>2025-09 = $30000.00</v>
+      </c>
+      <c r="H87" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Teens (8 a 12 años)</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Histórica - Teens (8 a 12 años) - 2025 - $25.000</v>
+      </c>
+      <c r="D88" t="str">
+        <v>25000.00</v>
+      </c>
+      <c r="E88" t="str">
+        <v>2025-11-01</v>
+      </c>
+      <c r="F88" t="str">
+        <v>2025-11-30</v>
+      </c>
+      <c r="G88" t="str">
+        <v>2025-11 = $25000.00</v>
+      </c>
+      <c r="H88" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Teens (8 a 12 años)</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Histórica - Teens (8 a 12 años) - 2026 - $30.000</v>
+      </c>
+      <c r="D89" t="str">
+        <v>30000.00</v>
+      </c>
+      <c r="E89" t="str">
+        <v>2026-01-01</v>
+      </c>
+      <c r="F89" t="str">
+        <v>2026-01-31</v>
+      </c>
+      <c r="G89" t="str">
+        <v>2026-01 = $30000.00</v>
+      </c>
+      <c r="H89" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Teens (8 a 12 años)</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Histórica - Teens (8 a 12 años) - 2026 - $15.000</v>
+      </c>
+      <c r="D90" t="str">
+        <v>15000.00</v>
+      </c>
+      <c r="E90" t="str">
+        <v>2026-02-01</v>
+      </c>
+      <c r="F90" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="G90" t="str">
+        <v>2026-02 = $15000.00</v>
+      </c>
+      <c r="H90" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+      </c>
+      <c r="B91" t="str">
+        <v>Teens (8 a 12 años)</v>
+      </c>
+      <c r="C91" t="str">
+        <v>Histórica - Teens (8 a 12 años) - 2026 - $30.000</v>
+      </c>
+      <c r="D91" t="str">
+        <v>30000.00</v>
+      </c>
+      <c r="E91" t="str">
+        <v>2026-03-01</v>
+      </c>
+      <c r="F91" t="str">
+        <v>2026-07-31</v>
+      </c>
+      <c r="G91" t="str">
+        <v>2026-03 = $30000.00 | 2026-05 = $30000.00</v>
+      </c>
+      <c r="H91" t="str">
+        <v>2026-07 ($15000.00)</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>da4d15d9-c846-4098-8640-e95fd97c604f</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Teens (8 a 12 años)</v>
+      </c>
+      <c r="C92" t="str">
+        <v>Histórica - Teens (8 a 12 años) - 2026 - $40.000</v>
+      </c>
+      <c r="D92" t="str">
+        <v>40000.00</v>
+      </c>
+      <c r="E92" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="F92" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G92" t="str">
+        <v>2026-08 = $40000.00</v>
+      </c>
+      <c r="H92" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
         <v>5e8e8fd7-a08b-4443-8ba0-30ee263ffa1b</v>
       </c>
-      <c r="B74" t="str">
+      <c r="B93" t="str">
         <v>Zumba - Profe Joselo</v>
       </c>
-      <c r="C74" t="str">
+      <c r="C93" t="str">
+        <v>Histórica - Zumba - Profe Joselo - 2026 - $30.000</v>
+      </c>
+      <c r="D93" t="str">
+        <v>30000.00</v>
+      </c>
+      <c r="E93" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="F93" t="str">
+        <v>2026-07-31</v>
+      </c>
+      <c r="G93" t="str">
+        <v>2026-05 = $30000.00</v>
+      </c>
+      <c r="H93" t="str">
+        <v>2026-07 ($15000.00)</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>5e8e8fd7-a08b-4443-8ba0-30ee263ffa1b</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Zumba - Profe Joselo</v>
+      </c>
+      <c r="C94" t="str">
         <v>Histórica - Zumba - Profe Joselo - 2026 - $40.000</v>
       </c>
-      <c r="D74" t="str">
+      <c r="D94" t="str">
         <v>40000.00</v>
       </c>
-      <c r="E74" t="str">
+      <c r="E94" t="str">
         <v>2026-08-01</v>
       </c>
-      <c r="F74" t="str">
+      <c r="F94" t="str">
         <v>2026-08-31</v>
       </c>
-      <c r="G74" t="str">
+      <c r="G94" t="str">
         <v>2026-08 = $40000.00</v>
       </c>
-      <c r="H74" t="str">
+      <c r="H94" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H74"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H94"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2727,7 +3247,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2774,7 +3294,7 @@
         <v>Tarifas consolidadas</v>
       </c>
       <c r="B6">
-        <v>73</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7">
@@ -2801,9 +3321,17 @@
         <v>0</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Períodos confirmados por PO</v>
+      </c>
+      <c r="B10">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>